<commit_message>
Major! Keep. Case studies. Update
</commit_message>
<xml_diff>
--- a/data/OP2/case18_1/case18_operational_data.xlsx
+++ b/data/OP2/case18_1/case18_operational_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/micaelsimoes/PycharmProjects/shared-resources-planning/data/OP2/case18_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD05FFE5-EBDE-3C4C-BE5A-5ABB27F7733B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93425957-102A-BA48-96D5-0963A2DEC5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1120" yWindow="620" windowWidth="50080" windowHeight="28180" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1120" yWindow="620" windowWidth="50080" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Characterization" sheetId="2" r:id="rId1"/>
@@ -454,16 +454,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <f>E2*3.5</f>
-        <v>0.70000000000000007</v>
+        <f>E2*4</f>
+        <v>0.8</v>
       </c>
       <c r="C2" s="1">
-        <f>F2*2</f>
-        <v>0.24</v>
+        <f>F2*2.5</f>
+        <v>0.3</v>
       </c>
       <c r="D2" s="2">
         <f>$B2/SUM($B$2:$B$1048576)</f>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E2" s="1">
         <v>0.2</v>
@@ -477,16 +477,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1">
-        <f t="shared" ref="B3:B31" si="0">E3*3.5</f>
-        <v>1.4000000000000001</v>
+        <f t="shared" ref="B3:B31" si="0">E3*4</f>
+        <v>1.6</v>
       </c>
       <c r="C3" s="1">
-        <f t="shared" ref="C3:C31" si="1">F3*2</f>
-        <v>0.5</v>
+        <f t="shared" ref="C3:C31" si="1">F3*2.5</f>
+        <v>0.625</v>
       </c>
       <c r="D3" s="2">
         <f t="shared" ref="D3:D31" si="2">$B3/SUM($B$2:$B$1048576)</f>
-        <v>1.7241379310344827E-2</v>
+        <v>1.886792452830189E-2</v>
       </c>
       <c r="E3" s="1">
         <v>0.4</v>
@@ -501,15 +501,15 @@
       </c>
       <c r="B4" s="1">
         <f t="shared" si="0"/>
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1">
         <f t="shared" si="1"/>
-        <v>1.86</v>
+        <v>2.3250000000000002</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="2"/>
-        <v>6.4655172413793108E-2</v>
+        <v>7.0754716981132074E-2</v>
       </c>
       <c r="E4" s="1">
         <v>1.5</v>
@@ -524,21 +524,21 @@
       </c>
       <c r="B5" s="1">
         <f t="shared" si="0"/>
-        <v>10.5</v>
+        <v>8</v>
       </c>
       <c r="C5" s="1">
         <f t="shared" si="1"/>
-        <v>4.5199999999999996</v>
+        <v>3.75</v>
       </c>
       <c r="D5" s="2">
         <f t="shared" si="2"/>
-        <v>0.12931034482758622</v>
+        <v>9.4339622641509441E-2</v>
       </c>
       <c r="E5" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="1">
-        <v>2.2599999999999998</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -547,15 +547,15 @@
       </c>
       <c r="B6" s="1">
         <f t="shared" si="0"/>
-        <v>2.8000000000000003</v>
+        <v>3.2</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="D6" s="2">
         <f t="shared" si="2"/>
-        <v>3.4482758620689655E-2</v>
+        <v>3.7735849056603779E-2</v>
       </c>
       <c r="E6" s="1">
         <v>0.8</v>
@@ -570,15 +570,15 @@
       </c>
       <c r="B7" s="1">
         <f t="shared" si="0"/>
-        <v>0.70000000000000007</v>
+        <v>0.8</v>
       </c>
       <c r="C7" s="1">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="2"/>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E7" s="1">
         <v>0.2</v>
@@ -593,15 +593,15 @@
       </c>
       <c r="B8" s="1">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="1">
         <f t="shared" si="1"/>
-        <v>1.24</v>
+        <v>1.55</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="2"/>
-        <v>4.3103448275862065E-2</v>
+        <v>4.716981132075472E-2</v>
       </c>
       <c r="E8" s="1">
         <v>1</v>
@@ -616,15 +616,15 @@
       </c>
       <c r="B9" s="1">
         <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="C9" s="1">
         <f t="shared" si="1"/>
-        <v>0.62</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="D9" s="2">
         <f t="shared" si="2"/>
-        <v>2.1551724137931032E-2</v>
+        <v>2.358490566037736E-2</v>
       </c>
       <c r="E9" s="1">
         <v>0.5</v>
@@ -639,15 +639,15 @@
       </c>
       <c r="B10" s="1">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="C10" s="1">
         <f t="shared" si="1"/>
-        <v>1.24</v>
+        <v>1.55</v>
       </c>
       <c r="D10" s="2">
         <f t="shared" si="2"/>
-        <v>4.3103448275862065E-2</v>
+        <v>4.716981132075472E-2</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
@@ -662,15 +662,15 @@
       </c>
       <c r="B11" s="1">
         <f t="shared" si="0"/>
-        <v>1.05</v>
+        <v>1.2</v>
       </c>
       <c r="C11" s="1">
         <f t="shared" si="1"/>
-        <v>0.38</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="D11" s="2">
         <f t="shared" si="2"/>
-        <v>1.2931034482758621E-2</v>
+        <v>1.4150943396226415E-2</v>
       </c>
       <c r="E11" s="1">
         <v>0.3</v>
@@ -685,15 +685,15 @@
       </c>
       <c r="B12" s="1">
         <f t="shared" si="0"/>
-        <v>0.70000000000000007</v>
+        <v>0.8</v>
       </c>
       <c r="C12" s="1">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D12" s="2">
         <f t="shared" si="2"/>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E12" s="1">
         <v>0.2</v>
@@ -708,15 +708,15 @@
       </c>
       <c r="B13" s="1">
         <f t="shared" si="0"/>
-        <v>2.8000000000000003</v>
+        <v>3.2</v>
       </c>
       <c r="C13" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="D13" s="2">
         <f t="shared" si="2"/>
-        <v>3.4482758620689655E-2</v>
+        <v>3.7735849056603779E-2</v>
       </c>
       <c r="E13" s="1">
         <v>0.8</v>
@@ -731,15 +731,15 @@
       </c>
       <c r="B14" s="1">
         <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="C14" s="1">
         <f t="shared" si="1"/>
-        <v>0.62</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="D14" s="2">
         <f t="shared" si="2"/>
-        <v>2.1551724137931032E-2</v>
+        <v>2.358490566037736E-2</v>
       </c>
       <c r="E14" s="1">
         <v>0.5</v>
@@ -754,15 +754,15 @@
       </c>
       <c r="B15" s="1">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="C15" s="1">
         <f t="shared" si="1"/>
-        <v>1.24</v>
+        <v>1.55</v>
       </c>
       <c r="D15" s="2">
         <f t="shared" si="2"/>
-        <v>4.3103448275862065E-2</v>
+        <v>4.716981132075472E-2</v>
       </c>
       <c r="E15" s="1">
         <v>1</v>
@@ -777,15 +777,15 @@
       </c>
       <c r="B16" s="1">
         <f t="shared" si="0"/>
-        <v>0.70000000000000007</v>
+        <v>0.8</v>
       </c>
       <c r="C16" s="1">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D16" s="2">
         <f t="shared" si="2"/>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E16" s="1">
         <v>0.2</v>
@@ -800,15 +800,15 @@
       </c>
       <c r="B17" s="1">
         <f t="shared" si="0"/>
-        <v>0.70000000000000007</v>
+        <v>0.8</v>
       </c>
       <c r="C17" s="1">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D17" s="2">
         <f>$B17/SUM($B$2:$B$1048576)</f>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E17" s="1">
         <v>0.2</v>
@@ -823,15 +823,15 @@
       </c>
       <c r="B18" s="1">
         <f t="shared" si="0"/>
-        <v>1.4000000000000001</v>
+        <v>1.6</v>
       </c>
       <c r="C18" s="1">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
       <c r="D18" s="2">
         <f t="shared" si="2"/>
-        <v>1.7241379310344827E-2</v>
+        <v>1.886792452830189E-2</v>
       </c>
       <c r="E18" s="1">
         <v>0.4</v>
@@ -846,15 +846,15 @@
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="C19" s="1">
         <f t="shared" si="1"/>
-        <v>1.86</v>
+        <v>2.3250000000000002</v>
       </c>
       <c r="D19" s="2">
         <f t="shared" si="2"/>
-        <v>6.4655172413793108E-2</v>
+        <v>7.0754716981132074E-2</v>
       </c>
       <c r="E19" s="1">
         <v>1.5</v>
@@ -869,21 +869,21 @@
       </c>
       <c r="B20" s="1">
         <f t="shared" si="0"/>
-        <v>10.5</v>
+        <v>8</v>
       </c>
       <c r="C20" s="1">
         <f t="shared" si="1"/>
-        <v>4.5199999999999996</v>
+        <v>3.75</v>
       </c>
       <c r="D20" s="2">
         <f t="shared" si="2"/>
-        <v>0.12931034482758622</v>
+        <v>9.4339622641509441E-2</v>
       </c>
       <c r="E20" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" s="1">
-        <v>2.2599999999999998</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -892,15 +892,15 @@
       </c>
       <c r="B21" s="1">
         <f t="shared" si="0"/>
-        <v>2.8000000000000003</v>
+        <v>3.2</v>
       </c>
       <c r="C21" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="D21" s="2">
         <f t="shared" si="2"/>
-        <v>3.4482758620689655E-2</v>
+        <v>3.7735849056603779E-2</v>
       </c>
       <c r="E21" s="1">
         <v>0.8</v>
@@ -915,15 +915,15 @@
       </c>
       <c r="B22" s="1">
         <f t="shared" si="0"/>
-        <v>0.70000000000000007</v>
+        <v>0.8</v>
       </c>
       <c r="C22" s="1">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D22" s="2">
         <f t="shared" si="2"/>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E22" s="1">
         <v>0.2</v>
@@ -938,15 +938,15 @@
       </c>
       <c r="B23" s="1">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="C23" s="1">
         <f t="shared" si="1"/>
-        <v>1.24</v>
+        <v>1.55</v>
       </c>
       <c r="D23" s="2">
         <f t="shared" si="2"/>
-        <v>4.3103448275862065E-2</v>
+        <v>4.716981132075472E-2</v>
       </c>
       <c r="E23" s="1">
         <v>1</v>
@@ -961,15 +961,15 @@
       </c>
       <c r="B24" s="1">
         <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="C24" s="1">
         <f t="shared" si="1"/>
-        <v>0.62</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="D24" s="2">
         <f t="shared" si="2"/>
-        <v>2.1551724137931032E-2</v>
+        <v>2.358490566037736E-2</v>
       </c>
       <c r="E24" s="1">
         <v>0.5</v>
@@ -984,15 +984,15 @@
       </c>
       <c r="B25" s="1">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="C25" s="1">
         <f t="shared" si="1"/>
-        <v>1.24</v>
+        <v>1.55</v>
       </c>
       <c r="D25" s="2">
         <f t="shared" si="2"/>
-        <v>4.3103448275862065E-2</v>
+        <v>4.716981132075472E-2</v>
       </c>
       <c r="E25" s="1">
         <v>1</v>
@@ -1007,15 +1007,15 @@
       </c>
       <c r="B26" s="1">
         <f t="shared" si="0"/>
-        <v>1.05</v>
+        <v>1.2</v>
       </c>
       <c r="C26" s="1">
         <f t="shared" si="1"/>
-        <v>0.38</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="D26" s="2">
         <f t="shared" si="2"/>
-        <v>1.2931034482758621E-2</v>
+        <v>1.4150943396226415E-2</v>
       </c>
       <c r="E26" s="1">
         <v>0.3</v>
@@ -1030,15 +1030,15 @@
       </c>
       <c r="B27" s="1">
         <f t="shared" si="0"/>
-        <v>0.70000000000000007</v>
+        <v>0.8</v>
       </c>
       <c r="C27" s="1">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D27" s="2">
         <f t="shared" si="2"/>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E27" s="1">
         <v>0.2</v>
@@ -1053,15 +1053,15 @@
       </c>
       <c r="B28" s="1">
         <f t="shared" si="0"/>
-        <v>2.8000000000000003</v>
+        <v>3.2</v>
       </c>
       <c r="C28" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="D28" s="2">
         <f t="shared" si="2"/>
-        <v>3.4482758620689655E-2</v>
+        <v>3.7735849056603779E-2</v>
       </c>
       <c r="E28" s="1">
         <v>0.8</v>
@@ -1076,15 +1076,15 @@
       </c>
       <c r="B29" s="1">
         <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="C29" s="1">
         <f t="shared" si="1"/>
-        <v>0.62</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="D29" s="2">
         <f t="shared" si="2"/>
-        <v>2.1551724137931032E-2</v>
+        <v>2.358490566037736E-2</v>
       </c>
       <c r="E29" s="1">
         <v>0.5</v>
@@ -1099,15 +1099,15 @@
       </c>
       <c r="B30" s="1">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="C30" s="1">
         <f t="shared" si="1"/>
-        <v>1.24</v>
+        <v>1.55</v>
       </c>
       <c r="D30" s="2">
         <f t="shared" si="2"/>
-        <v>4.3103448275862065E-2</v>
+        <v>4.716981132075472E-2</v>
       </c>
       <c r="E30" s="1">
         <v>1</v>
@@ -1122,15 +1122,15 @@
       </c>
       <c r="B31" s="1">
         <f t="shared" si="0"/>
-        <v>0.70000000000000007</v>
+        <v>0.8</v>
       </c>
       <c r="C31" s="1">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D31" s="2">
         <f t="shared" si="2"/>
-        <v>8.6206896551724137E-3</v>
+        <v>9.4339622641509448E-3</v>
       </c>
       <c r="E31" s="1">
         <v>0.2</v>

</xml_diff>